<commit_message>
modified shopping data dictionary
</commit_message>
<xml_diff>
--- a/data/reference-tables/data_dictionary_e-shop-clothing-2008-processed.xlsx
+++ b/data/reference-tables/data_dictionary_e-shop-clothing-2008-processed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxwe\Desktop\inst414-final-project-maxwell-liu\data\reference-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E67EAC-F4ED-4F64-9EDA-8329C5F3DCD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E85BC94-472D-465E-AA98-885FB74B0D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17304" windowHeight="8892" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3156" yWindow="828" windowWidth="17304" windowHeight="8892" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -108,9 +108,6 @@
     <t>Click order in the session</t>
   </si>
   <si>
-    <t>Country of origin by IP</t>
-  </si>
-  <si>
     <t>Unique session identifier</t>
   </si>
   <si>
@@ -145,6 +142,9 @@
   </si>
   <si>
     <t>None</t>
+  </si>
+  <si>
+    <t>Country of origin by number</t>
   </si>
 </sst>
 </file>
@@ -496,7 +496,7 @@
         <v>2008</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -513,7 +513,7 @@
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -530,7 +530,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -547,7 +547,7 @@
         <v>3</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -555,7 +555,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
@@ -564,7 +564,7 @@
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -572,7 +572,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -581,7 +581,7 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -589,7 +589,7 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>21</v>
@@ -598,7 +598,7 @@
         <v>2</v>
       </c>
       <c r="E8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -606,16 +606,16 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -623,7 +623,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
         <v>21</v>
@@ -632,7 +632,7 @@
         <v>10</v>
       </c>
       <c r="E10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -640,7 +640,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
         <v>21</v>
@@ -649,7 +649,7 @@
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -657,7 +657,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
         <v>21</v>
@@ -666,7 +666,7 @@
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -674,7 +674,7 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -683,7 +683,7 @@
         <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -691,7 +691,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
         <v>22</v>
@@ -700,7 +700,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -708,7 +708,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
@@ -717,7 +717,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>